<commit_message>
app aizpildīti dienas ieraksti - jauni dati json failu formātā + papildināts atziņu žurnāls
</commit_message>
<xml_diff>
--- a/Atzinu zurnals 1 .xlsx
+++ b/Atzinu zurnals 1 .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\KURSI 2\1 ned\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73106861-0EBA-4764-B353-2DE17021FC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A19319-F1CA-430E-972D-1713AE1ED3F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D6D6D45E-E888-4B90-B661-1ADACB5382D8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D6D6D45E-E888-4B90-B661-1ADACB5382D8}"/>
   </bookViews>
   <sheets>
     <sheet name="Žurnāls" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="114">
   <si>
     <t>Atziņu žurnāls</t>
   </si>
@@ -471,31 +471,33 @@
     <t>Datubāzes pārskats</t>
   </si>
   <si>
-    <t>Datubāzē glabājas divas tabulas:
+    <t>Datubāzē "app.db"glabājas divas tabulas:
 - daily entries (glabā id, user id - datumu un dienas pierakstus 3 labas lietas un 1-3 lietas kuras neizdevās)
 - users (glabā id, lietotāvārdu, paroli un izveidošanas datumu.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Datubāzes pārskats </t>
-  </si>
-  <si>
-    <t>daily_entries kolonnas 
-    -id 
-    -user id
-    -date
-    -positive_Things
-    -negative_Things
-    -gratitude
-    -emotions
-    -notes
-    -dialy_entry
-    -sync_satus
-    -updatead_ad 
-Users kolonnas 
-    -id 
-    -username
-    -password_hash
-    -created_at</t>
+    <t xml:space="preserve">Izpētīt kādas tabulas pastāv </t>
+  </si>
+  <si>
+    <t xml:space="preserve">izskaidro iesācēju līmenī - tabulas nosaukumus. Kādus datus tā glabā, kādas kolonnas tajā ir. kādi ir datu tipi kolonnās. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">`INTEGER` - tikai vesaliem skaitļiem. `VARCHAR` - noteikta garuma īsiem vārdiem teksts.  va `TEXT` - jebkāda garuma tekstiem. `DATE / DATETIME` - kalendārs, datums pulksteņi.  </t>
+  </si>
+  <si>
+    <t>izskaidro iesācēju līmenī kā tabulas ir sasistītas. Kuras divas tabulas ir sasitīTAS. Kura kolonna ir ārējā atslēga (Foreign key). Kāda veida attiecība tā ir -one-to many, one-to-one, many-to-one. kāpēc ši saistība pastāv. ko tā nozīmē lietotnes kontekstā?</t>
+  </si>
+  <si>
+    <t>Izpētīt attiecības starp tabulām.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Domāju, ka tabulas sastāv tikai no skaitļiem </t>
+  </si>
+  <si>
+    <t>Domāju, ka visas tabulas savā starpā ir sasitītas.</t>
+  </si>
+  <si>
+    <t>Savā starpā ir saistītas `users`(Lietotāji) un tabula `daily_entries`(dienas ieraksti).  (Foreign Key) ir `user_id`, atrodas tabulā `daily_entries`. Attiecības "One-to-Many" = viens pret daudziem attiecība, jo lietotājs (''users) var veikt daudz ierakstu 'daily_entries' tabulā.</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1286,7 @@
     <col min="5" max="5" width="52.33203125" style="7" customWidth="1"/>
     <col min="6" max="6" width="48.33203125" style="7" customWidth="1"/>
     <col min="7" max="7" width="51" style="7" customWidth="1"/>
-    <col min="8" max="8" width="44.44140625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="48.21875" style="7" customWidth="1"/>
     <col min="9" max="9" width="21.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="2"/>
   </cols>
@@ -1996,9 +1998,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:9" ht="248.4">
+    <row r="32" spans="2:9" ht="69">
       <c r="B32" s="13">
-        <v>46131</v>
+        <v>46133</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>19</v>
@@ -2009,26 +2011,44 @@
       <c r="E32" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="F32" s="8"/>
+      <c r="F32" s="8" t="s">
+        <v>111</v>
+      </c>
       <c r="G32" s="8" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I32" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="2:9">
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="82.8">
+      <c r="B33" s="13">
+        <v>46133</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="I33" s="8">
+        <v>30</v>
+      </c>
     </row>
     <row r="34" spans="2:9">
       <c r="B34" s="8"/>
@@ -9787,12 +9807,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokuments" ma:contentTypeID="0x01010005545F18E44C8342BA252CB175FF88D8" ma:contentTypeVersion="7" ma:contentTypeDescription="Izveidot jaunu dokumentu." ma:contentTypeScope="" ma:versionID="65c4e2c089a594a7e1f8c8c39588e85e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="655e3d82-d0a4-453c-95d0-0de2a489e81f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="806de7c62a768292a734b69de171ceb4" ns2:_="">
     <xsd:import namespace="655e3d82-d0a4-453c-95d0-0de2a489e81f"/>
@@ -9954,6 +9968,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40D2E0B9-1A30-4C03-B4DA-DFF248A05241}">
   <ds:schemaRefs>
@@ -9963,15 +9983,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{328DC1B4-4C62-49A4-9AE8-0ADDF1506538}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B40AF704-B88D-4751-8BBA-30506D95E0B4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9987,4 +9998,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{328DC1B4-4C62-49A4-9AE8-0ADDF1506538}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>